<commit_message>
Vailid Palindrome 1 & 2 Is Subsequence and changes in excel
</commit_message>
<xml_diff>
--- a/DSA Final Sheet Algomaster600.xlsx
+++ b/DSA Final Sheet Algomaster600.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Surya\Documents\GitHub\DSA600\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89BC71E-41D1-4068-B1AE-BFB0EB76026D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1692C007-C571-4480-A167-09FF10D1231A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -427,6 +427,52 @@
         </r>
       </text>
     </comment>
+    <comment ref="G22" authorId="0" shapeId="0" xr:uid="{88E35B03-B88B-45A4-9F91-2BFF8995E93C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>placed variables at the start incremented if both same and incremented only right if not same 
+check if variable = size
+return true else false</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G23" authorId="0" shapeId="0" xr:uid="{F772FC85-A235-4C0F-A96F-5CF286A4D081}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>used 2 pointer approach did tolower on both sides checked if isalnum then returned if true else false</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G24" authorId="0" shapeId="0" xr:uid="{77DAA129-0FC9-453B-9176-58DBB2C56281}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>check for palindrome using 2 pointer then at first mistake made another function which check for palindrome 
+1) start to end (excluding end)
+2) start to end (excluding start)</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="G54" authorId="0" shapeId="0" xr:uid="{33A35E6F-F8FA-4B1C-9AE0-695776DBD5F4}">
       <text>
         <r>
@@ -449,7 +495,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1933" uniqueCount="694">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1948" uniqueCount="695">
   <si>
     <t>Category</t>
   </si>
@@ -2531,6 +2577,9 @@
   </si>
   <si>
     <t>Single check from the end</t>
+  </si>
+  <si>
+    <t>2 Variables on both string start</t>
   </si>
 </sst>
 </file>
@@ -3823,12 +3872,22 @@
       <c r="D22" s="8" t="s">
         <v>679</v>
       </c>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
+      <c r="E22" s="11" t="s">
+        <v>673</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>674</v>
+      </c>
       <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
+      <c r="H22" s="8" t="s">
+        <v>677</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>684</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>694</v>
+      </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
     </row>
@@ -3845,12 +3904,22 @@
       <c r="D23" s="8" t="s">
         <v>679</v>
       </c>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
+      <c r="E23" s="11" t="s">
+        <v>673</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>674</v>
+      </c>
       <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
+      <c r="H23" s="8" t="s">
+        <v>677</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>684</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>680</v>
+      </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8"/>
     </row>
@@ -3867,12 +3936,22 @@
       <c r="D24" s="8" t="s">
         <v>679</v>
       </c>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
+      <c r="E24" s="11" t="s">
+        <v>673</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>674</v>
+      </c>
       <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
+      <c r="H24" s="8" t="s">
+        <v>677</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>684</v>
+      </c>
+      <c r="J24" s="8" t="s">
+        <v>680</v>
+      </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8"/>
     </row>

</xml_diff>

<commit_message>
1) Valid Anagram 2) Rotate String Sheet updation
</commit_message>
<xml_diff>
--- a/DSA Final Sheet Algomaster600.xlsx
+++ b/DSA Final Sheet Algomaster600.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Surya\Documents\GitHub\DSA600\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1692C007-C571-4480-A167-09FF10D1231A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B843472-2939-4C26-85CF-E2245B7475A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -473,6 +473,22 @@
         </r>
       </text>
     </comment>
+    <comment ref="G25" authorId="0" shapeId="0" xr:uid="{6C604F96-8D7D-42EE-9EDF-9ECB3350E2CD}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>check for palindrome using 2 pointer then at first mistake made another function which check for palindrome 
+1) start to end (excluding end)
+2) start to end (excluding start)</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="G54" authorId="0" shapeId="0" xr:uid="{33A35E6F-F8FA-4B1C-9AE0-695776DBD5F4}">
       <text>
         <r>
@@ -495,7 +511,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1948" uniqueCount="695">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1953" uniqueCount="696">
   <si>
     <t>Category</t>
   </si>
@@ -2580,6 +2596,9 @@
   </si>
   <si>
     <t>2 Variables on both string start</t>
+  </si>
+  <si>
+    <t>frequency counting using a fixed-size array</t>
   </si>
 </sst>
 </file>
@@ -3968,12 +3987,22 @@
       <c r="D25" s="8" t="s">
         <v>679</v>
       </c>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
+      <c r="E25" s="11" t="s">
+        <v>673</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>674</v>
+      </c>
       <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
+      <c r="H25" s="8" t="s">
+        <v>677</v>
+      </c>
+      <c r="I25" s="8" t="s">
+        <v>684</v>
+      </c>
+      <c r="J25" t="s">
+        <v>695</v>
+      </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8"/>
     </row>

</xml_diff>